<commit_message>
wip: sesion base de datos (scripts DB, ratios, valuacion, flags, docs)
</commit_message>
<xml_diff>
--- a/scripts/tickets/datos/reporte_tickets.xlsx
+++ b/scripts/tickets/datos/reporte_tickets.xlsx
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -507,7 +507,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
@@ -701,19 +701,19 @@
         <v>10.64831038798498</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2233362039616473</v>
+        <v>0.1717807657942223</v>
       </c>
       <c r="K3" t="n">
         <v>0.2931367144432194</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1225162252429885</v>
+        <v>-0.0057633415570256</v>
       </c>
       <c r="M3" t="n">
-        <v>0.6199362767410105</v>
+        <v>0.6231270730870411</v>
       </c>
       <c r="N3" t="n">
-        <v>0.8928083750568958</v>
+        <v>0.8974036371954707</v>
       </c>
       <c r="O3" t="n">
         <v>0.1820008856490786</v>
@@ -770,34 +770,34 @@
         <v>351.4299926757812</v>
       </c>
       <c r="H4" t="n">
-        <v>24.79288237785307</v>
+        <v>24.50998923277244</v>
       </c>
       <c r="I4" t="n">
-        <v>14.17463235294118</v>
+        <v>14.33823529411765</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.0020687637475209</v>
+        <v>0.0294123386111588</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2098174199341514</v>
+        <v>0.2095647501343363</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4071572813123167</v>
+        <v>0.1050291183127298</v>
       </c>
       <c r="M4" t="n">
-        <v>4.023513722187127</v>
+        <v>3.706867563372995</v>
       </c>
       <c r="N4" t="n">
-        <v>4.545448164525865</v>
+        <v>4.187726332126228</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1217807045239276</v>
+        <v>0.1292529279990378</v>
       </c>
       <c r="P4" t="n">
-        <v>0.1308329699084169</v>
+        <v>0.1388606225065012</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.6645052522370639</v>
+        <v>0.6670512820512821</v>
       </c>
       <c r="R4" t="n">
         <v>-0.1018682179424075</v>
@@ -845,30 +845,30 @@
         <v>163.1499938964844</v>
       </c>
       <c r="H5" t="n">
-        <v>18.25951966574026</v>
+        <v>18.21187232535416</v>
       </c>
       <c r="I5" t="n">
-        <v>8.935064935064934</v>
+        <v>8.958441558441558</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0326462051370326</v>
+        <v>0.0586623863271</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0776918299361978</v>
+        <v>0.076595933686443</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.1137583320461178</v>
+        <v>-0.08412793167586489</v>
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
-        <v>0.1295390490044549</v>
+        <v>0.1587235203200291</v>
       </c>
       <c r="P5" t="n">
-        <v>0.116798373610519</v>
+        <v>0.1431124372889136</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.4191860465116279</v>
+        <v>0.4222963177732676</v>
       </c>
       <c r="R5" t="n">
         <v>-0.1823694528117305</v>
@@ -916,30 +916,30 @@
         <v>342.5599975585937</v>
       </c>
       <c r="H6" t="n">
-        <v>21.69262054141931</v>
+        <v>20.94439913771794</v>
       </c>
       <c r="I6" t="n">
-        <v>15.79154518950437</v>
+        <v>16.35568513119534</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2216355977255029</v>
+        <v>0.3247166566380277</v>
       </c>
       <c r="K6" t="n">
-        <v>0.2622748402091807</v>
+        <v>0.2659082829719161</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.0221332739268453</v>
+        <v>0.2322739764278127</v>
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
-        <v>0.1725483853577012</v>
+        <v>0.154444983557065</v>
       </c>
       <c r="P6" t="n">
-        <v>0.3138027727121203</v>
+        <v>0.2808792674078867</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.2096372196067571</v>
+        <v>0.2090017825311943</v>
       </c>
       <c r="R6" t="n">
         <v>-0.1159513634109752</v>
@@ -987,26 +987,26 @@
         <v>57.72999954223633</v>
       </c>
       <c r="H7" t="n">
-        <v>14.03560495606339</v>
+        <v>13.49422593528938</v>
       </c>
       <c r="I7" t="n">
-        <v>4.113110886417257</v>
+        <v>4.278126053252444</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0316487739959585</v>
+        <v>0.1529664601415619</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2697595869032777</v>
+        <v>0.2756467052344469</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.0178545962584377</v>
+        <v>0.0924179029389951</v>
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
-        <v>0.0467730833524533</v>
+        <v>0.0449689597579806</v>
       </c>
       <c r="R7" t="n">
         <v>-0.0048267331046093</v>
@@ -1122,13 +1122,13 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="n">
-        <v>-0.0321354147625489</v>
+        <v>-0.0424450700106021</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.028245501285347</v>
+        <v>-0.0373071979434447</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.6720351390922401</v>
+        <v>0.7379209370424598</v>
       </c>
       <c r="R9" t="n">
         <v>-0.1918884717904159</v>
@@ -1231,31 +1231,31 @@
         <v>199.5899963378907</v>
       </c>
       <c r="H11" t="n">
-        <v>22.90908458236752</v>
+        <v>21.58987933270863</v>
       </c>
       <c r="I11" t="n">
-        <v>8.712264150943396</v>
+        <v>9.244609164420485</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.1806275146100012</v>
+        <v>-0.1873427038832538</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1307200776494853</v>
+        <v>0.1380542194135287</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.2171690760451573</v>
+        <v>-0.2325916897923189</v>
       </c>
       <c r="M11" t="n">
-        <v>1.736866817654532</v>
+        <v>1.918044287195754</v>
       </c>
       <c r="N11" t="n">
-        <v>1.736866817654532</v>
+        <v>1.918044287195754</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0972500818004637</v>
+        <v>0.1148952716960911</v>
       </c>
       <c r="P11" t="n">
-        <v>0.112841280496528</v>
+        <v>0.1333153591354777</v>
       </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="n">
@@ -1343,13 +1343,13 @@
         <v>7.63760610752229</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.09568240565897999</v>
+        <v>0.0817005123749574</v>
       </c>
       <c r="K13" t="n">
         <v>0.1678615429744793</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.1387912838643539</v>
+        <v>0.0426215328313133</v>
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -1408,28 +1408,28 @@
         <v>994.4500122070312</v>
       </c>
       <c r="H14" t="n">
-        <v>52.15208463026742</v>
+        <v>49.13703359351174</v>
       </c>
       <c r="I14" t="n">
-        <v>19.06826964362387</v>
+        <v>20.23829969944182</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1441846658152443</v>
+        <v>0.280675881138706</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1314119161402003</v>
+        <v>0.1332344003957317</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>2.288526056810557</v>
+        <v>2.19665092314298</v>
       </c>
       <c r="N14" t="n">
-        <v>2.699619771863118</v>
+        <v>2.591240875912409</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>0.3095023643323575</v>
+        <v>0.2946854778826774</v>
       </c>
       <c r="R14" t="n">
         <v>-0.0281835710693746</v>
@@ -1477,31 +1477,31 @@
         <v>91.87999725341795</v>
       </c>
       <c r="H15" t="n">
-        <v>34.69633479771426</v>
+        <v>35.42748361529062</v>
       </c>
       <c r="I15" t="n">
-        <v>2.648118246180599</v>
+        <v>2.593466650105577</v>
       </c>
       <c r="J15" t="n">
-        <v>0.0014503324204158</v>
+        <v>-0.0348268761167296</v>
       </c>
       <c r="K15" t="n">
-        <v>0.1046020998920616</v>
+        <v>0.1004087521038711</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.1196136122247047</v>
+        <v>0.1784250681692956</v>
       </c>
       <c r="M15" t="n">
-        <v>1.991615853658537</v>
+        <v>2.045668058455115</v>
       </c>
       <c r="N15" t="n">
-        <v>2.27489837398374</v>
+        <v>2.336638830897704</v>
       </c>
       <c r="O15" t="n">
-        <v>0.4551603206412826</v>
+        <v>0.4718186372745491</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4680577022153529</v>
+        <v>0.4851880473982483</v>
       </c>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="n">
@@ -1556,13 +1556,13 @@
         <v>2.999247554552295</v>
       </c>
       <c r="J16" t="n">
-        <v>1.736665239794279</v>
+        <v>-0.00691310538226</v>
       </c>
       <c r="K16" t="n">
         <v>0.196852467652191</v>
       </c>
       <c r="L16" t="n">
-        <v>1.857961475466744</v>
+        <v>-0.0723039642624444</v>
       </c>
       <c r="M16" t="n">
         <v>1.535759854945941</v>
@@ -1631,13 +1631,13 @@
         <v>17.65596160944998</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3675486498000304</v>
+        <v>0.163135712601582</v>
       </c>
       <c r="K17" t="n">
         <v>0.1009220770999936</v>
       </c>
       <c r="L17" t="n">
-        <v>0.1649563099137492</v>
+        <v>0.0808101932709159</v>
       </c>
       <c r="M17" t="n">
         <v>2.85927035600987</v>
@@ -1700,34 +1700,34 @@
         <v>109.4499969482422</v>
       </c>
       <c r="H18" t="n">
-        <v>24.62759655605449</v>
+        <v>24.47096311416178</v>
       </c>
       <c r="I18" t="n">
-        <v>4.444201312910285</v>
+        <v>4.472647702407002</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1527242657162066</v>
+        <v>-0.1126753524230532</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1829729729729729</v>
+        <v>0.1761461564977594</v>
       </c>
       <c r="L18" t="n">
-        <v>0.0143826098966357</v>
+        <v>-0.2437080647094097</v>
       </c>
       <c r="M18" t="n">
-        <v>2.876676602086438</v>
+        <v>2.861749444032617</v>
       </c>
       <c r="N18" t="n">
-        <v>3.435543964232489</v>
+        <v>3.417716827279466</v>
       </c>
       <c r="O18" t="n">
-        <v>0.118190060166488</v>
+        <v>0.1390422813813566</v>
       </c>
       <c r="P18" t="n">
-        <v>0.1335319862184561</v>
+        <v>0.1570909768134835</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.2614475627769572</v>
+        <v>0.2622309197651663</v>
       </c>
       <c r="R18" t="n">
         <v>-0.08264186415316339</v>
@@ -1808,27 +1808,31 @@
         <v>365.8800048828125</v>
       </c>
       <c r="H20" t="n">
-        <v>44.30578184127808</v>
+        <v>44.68569236923341</v>
       </c>
       <c r="I20" t="n">
-        <v>8.258064516129032</v>
-      </c>
-      <c r="J20" t="inlineStr"/>
+        <v>8.187855787476281</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.1194602644183211</v>
+      </c>
       <c r="K20" t="n">
-        <v>0.1898157234761749</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
+        <v>0.1786305679748302</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.260347072461309</v>
+      </c>
       <c r="M20" t="n">
-        <v>0.7352634792916413</v>
+        <v>0.651339655062687</v>
       </c>
       <c r="N20" t="n">
-        <v>0.7359818959014333</v>
+        <v>0.6519760707694265</v>
       </c>
       <c r="O20" t="n">
-        <v>0.1885479935627887</v>
+        <v>0.1935056844728235</v>
       </c>
       <c r="P20" t="n">
-        <v>-1.528297917104986</v>
+        <v>-1.568483063328424</v>
       </c>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="n">
@@ -1877,26 +1881,26 @@
         <v>240.0200042724609</v>
       </c>
       <c r="H21" t="n">
-        <v>27.92225200809845</v>
+        <v>26.75934752009502</v>
       </c>
       <c r="I21" t="n">
-        <v>8.596011675664505</v>
+        <v>8.969576111383773</v>
       </c>
       <c r="J21" t="n">
-        <v>0.1288813207301975</v>
+        <v>0.1068799587449211</v>
       </c>
       <c r="K21" t="n">
-        <v>0.2296435907489857</v>
+        <v>0.232612160732399</v>
       </c>
       <c r="L21" t="n">
-        <v>0.0290088475065926</v>
+        <v>0.0276741106319007</v>
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="n">
-        <v>0.3989964462730943</v>
+        <v>0.3991231404749233</v>
       </c>
       <c r="R21" t="n">
         <v>-0.1218352193743963</v>
@@ -1944,28 +1948,28 @@
         <v>1076.910034179688</v>
       </c>
       <c r="H22" t="n">
-        <v>19.31114872655704</v>
+        <v>18.35777565460172</v>
       </c>
       <c r="I22" t="n">
-        <v>55.76623376623377</v>
+        <v>58.66233766233766</v>
       </c>
       <c r="J22" t="n">
-        <v>-0.0197605325957489</v>
+        <v>0.1571173099479696</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
-        <v>-0.0888091654478886</v>
+        <v>0.07383843116313769</v>
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
-        <v>-0.1343309483506636</v>
+        <v>-0.1192643063398813</v>
       </c>
       <c r="P22" t="n">
-        <v>-0.1932312980847929</v>
+        <v>-0.1715583565231625</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.3072310200279459</v>
+        <v>0.3182421961478858</v>
       </c>
       <c r="R22" t="n">
         <v>-0.0427466362847221</v>
@@ -2046,34 +2050,34 @@
         <v>342.8599853515625</v>
       </c>
       <c r="H24" t="n">
-        <v>24.12323717223483</v>
+        <v>24.37114940123867</v>
       </c>
       <c r="I24" t="n">
-        <v>14.21285140562249</v>
+        <v>14.06827309236948</v>
       </c>
       <c r="J24" t="n">
-        <v>0.092019327145572</v>
+        <v>0.0357146389096865</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0859590850300273</v>
+        <v>0.08410968113714939</v>
       </c>
       <c r="L24" t="n">
-        <v>0.6720894126163077</v>
+        <v>-0.1851733643786972</v>
       </c>
       <c r="M24" t="n">
-        <v>2.02413538764137</v>
+        <v>2.032212942773687</v>
       </c>
       <c r="N24" t="n">
-        <v>2.121906244877889</v>
+        <v>2.130373966347143</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1998703987608857</v>
+        <v>0.226248992429391</v>
       </c>
       <c r="P24" t="n">
-        <v>0.1974210066192082</v>
+        <v>0.2234763332084426</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.6465103136479231</v>
+        <v>0.6555809306308878</v>
       </c>
       <c r="R24" t="n">
         <v>-0.1965788275300234</v>
@@ -2182,28 +2186,28 @@
         <v>6.423872180451128</v>
       </c>
       <c r="J26" t="n">
-        <v>0.3346601172544363</v>
+        <v>0.0183608813392091</v>
       </c>
       <c r="K26" t="n">
         <v>0.1088953797132235</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2902515731593249</v>
+        <v>-0.0026378341910429</v>
       </c>
       <c r="M26" t="n">
-        <v>3.37456647398844</v>
+        <v>3.319102749638205</v>
       </c>
       <c r="N26" t="n">
-        <v>3.861166579085654</v>
+        <v>3.797705189166839</v>
       </c>
       <c r="O26" t="n">
-        <v>0.1186459222302457</v>
+        <v>0.0906365565986126</v>
       </c>
       <c r="P26" t="n">
-        <v>0.1413746349603671</v>
+        <v>0.1079995828118481</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.7256766642282371</v>
+        <v>0.7376249695196293</v>
       </c>
       <c r="R26" t="n">
         <v>-0.0836489447961121</v>
@@ -2257,7 +2261,7 @@
         <v>2.751077586206896</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>0.06002507028689</v>
       </c>
       <c r="K27" t="n">
         <v>0.0444641830816657</v>
@@ -2324,30 +2328,34 @@
         <v>276.0599975585937</v>
       </c>
       <c r="H28" t="n">
-        <v>73.77465451996902</v>
+        <v>63.79138705052367</v>
       </c>
       <c r="I28" t="n">
-        <v>3.741935483870968</v>
-      </c>
-      <c r="J28" t="inlineStr"/>
+        <v>4.327543424317618</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.292133353575134</v>
+      </c>
       <c r="K28" t="n">
-        <v>0.1827435773145904</v>
-      </c>
-      <c r="L28" t="inlineStr"/>
+        <v>0.2022497970543894</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.2171468273098051</v>
+      </c>
       <c r="M28" t="n">
-        <v>1.309574924860455</v>
+        <v>1.176243733127651</v>
       </c>
       <c r="N28" t="n">
-        <v>1.582653499355947</v>
+        <v>1.421519475510991</v>
       </c>
       <c r="O28" t="n">
-        <v>0.1669388707419505</v>
+        <v>0.1931871208586094</v>
       </c>
       <c r="P28" t="n">
-        <v>0.2112800826812343</v>
+        <v>0.2445002214675919</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.1511936339522546</v>
+        <v>0.1307339449541284</v>
       </c>
       <c r="R28" t="n">
         <v>-0.0501324951981253</v>
@@ -2395,30 +2403,30 @@
         <v>262.9599914550781</v>
       </c>
       <c r="H29" t="n">
-        <v>23.6356437848423</v>
+        <v>23.28179046055742</v>
       </c>
       <c r="I29" t="n">
-        <v>11.12556923978166</v>
+        <v>11.29466360847843</v>
       </c>
       <c r="J29" t="n">
-        <v>-0.0308355144407896</v>
+        <v>0.1238620988134662</v>
       </c>
       <c r="K29" t="n">
-        <v>0.1568520026652846</v>
+        <v>0.1560563625545994</v>
       </c>
       <c r="L29" t="n">
-        <v>-0.08086061259275749</v>
+        <v>0.0557560801718681</v>
       </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="n">
-        <v>0.1261702704393336</v>
+        <v>0.1346254092036948</v>
       </c>
       <c r="P29" t="n">
-        <v>0.1223647890314557</v>
+        <v>0.1305649083426861</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.5904842820730671</v>
+        <v>0.5841547331225591</v>
       </c>
       <c r="R29" t="n">
         <v>-0.2090477103600323</v>
@@ -2588,28 +2596,24 @@
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
-        <v>-0.0525280346252213</v>
-      </c>
-      <c r="J33" t="n">
-        <v>-0.3831829137416396</v>
-      </c>
+        <v>-0.6244343891402715</v>
+      </c>
+      <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>-0.0050517472991126</v>
-      </c>
-      <c r="L33" t="n">
-        <v>-0.4375453743971594</v>
-      </c>
+        <v>-0.0590368841024496</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
-        <v>5.453002458152874</v>
+        <v>6.543756145526057</v>
       </c>
       <c r="N33" t="n">
-        <v>6.230364040735105</v>
+        <v>7.47661188369153</v>
       </c>
       <c r="O33" t="n">
-        <v>-0.0313269485184739</v>
+        <v>-0.0197431304160679</v>
       </c>
       <c r="P33" t="n">
-        <v>-0.0335814565761706</v>
+        <v>-0.0211639852618865</v>
       </c>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="n">
@@ -2713,29 +2717,29 @@
         <v>241</v>
       </c>
       <c r="H35" t="n">
-        <v>21.98527085509625</v>
+        <v>28.0082319391635</v>
       </c>
       <c r="I35" t="n">
-        <v>10.96188450842467</v>
+        <v>8.60461311958122</v>
       </c>
       <c r="J35" t="n">
-        <v>0.1958542464109653</v>
+        <v>0.148906754567174</v>
       </c>
       <c r="K35" t="n">
-        <v>0.2845646704107524</v>
+        <v>0.21834333035844</v>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="n">
-        <v>1.424328876362011</v>
+        <v>1.404630351513508</v>
       </c>
       <c r="N35" t="n">
-        <v>2.093218299934692</v>
+        <v>2.064269007830243</v>
       </c>
       <c r="O35" t="n">
-        <v>0.1606373956158664</v>
+        <v>0.1450287056367432</v>
       </c>
       <c r="P35" t="n">
-        <v>0.1636100867138443</v>
+        <v>0.1477125485896541</v>
       </c>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="n">
@@ -2784,26 +2788,26 @@
         <v>333.4500122070312</v>
       </c>
       <c r="H36" t="n">
-        <v>15.89978129304386</v>
+        <v>15.40010396111252</v>
       </c>
       <c r="I36" t="n">
-        <v>20.97198735387104</v>
+        <v>21.65245202558636</v>
       </c>
       <c r="J36" t="n">
-        <v>0.1251623775466843</v>
+        <v>0.1765495483894246</v>
       </c>
       <c r="K36" t="n">
-        <v>0.31268258727192</v>
+        <v>0.3228279993641989</v>
       </c>
       <c r="L36" t="n">
-        <v>0.0360606470060915</v>
+        <v>0.0967436141444195</v>
       </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="n">
-        <v>0.2914212592904221</v>
+        <v>0.2916178542929422</v>
       </c>
       <c r="R36" t="n">
         <v>-0.0137241095007796</v>
@@ -2851,9 +2855,7 @@
         <v>99.91000366210938</v>
       </c>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="n">
-        <v>-1.516431555349548</v>
-      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -2969,28 +2971,28 @@
         <v>6.359543817527011</v>
       </c>
       <c r="J39" t="n">
-        <v>0.0527046357706644</v>
+        <v>-0.0244570588263157</v>
       </c>
       <c r="K39" t="n">
         <v>0.1279898526214061</v>
       </c>
       <c r="L39" t="n">
-        <v>-0.0649701591488699</v>
+        <v>-0.1206483844563919</v>
       </c>
       <c r="M39" t="n">
-        <v>2.345373891001268</v>
+        <v>2.27543805717799</v>
       </c>
       <c r="N39" t="n">
-        <v>2.843472750316857</v>
+        <v>2.758684291423302</v>
       </c>
       <c r="O39" t="n">
-        <v>0.1781909110676234</v>
+        <v>0.1997173298543161</v>
       </c>
       <c r="P39" t="n">
-        <v>0.1602463824794681</v>
+        <v>0.1796050058662495</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.7833883907503539</v>
+        <v>0.7895233600755073</v>
       </c>
       <c r="R39" t="n">
         <v>-0.2235559570493859</v>
@@ -3038,34 +3040,34 @@
         <v>80.59999847412109</v>
       </c>
       <c r="H40" t="n">
-        <v>26.52844994410303</v>
+        <v>25.37832226971451</v>
       </c>
       <c r="I40" t="n">
-        <v>3.038247566063978</v>
+        <v>3.175938803894298</v>
       </c>
       <c r="J40" t="n">
-        <v>0.1048953322154568</v>
+        <v>0.1117422496891589</v>
       </c>
       <c r="K40" t="n">
-        <v>0.2733985523873094</v>
+        <v>0.2780009739469199</v>
       </c>
       <c r="L40" t="n">
-        <v>0.0492323851764846</v>
+        <v>0.0937787743535141</v>
       </c>
       <c r="M40" t="n">
-        <v>2.463948150148528</v>
+        <v>2.353214262686182</v>
       </c>
       <c r="N40" t="n">
-        <v>2.718133945449635</v>
+        <v>2.595976529756916</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0755179740193072</v>
+        <v>0.1791270373169445</v>
       </c>
       <c r="P40" t="n">
-        <v>0.0836386607706885</v>
+        <v>0.198389134554643</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.6697947661554894</v>
+        <v>0.8007444712064813</v>
       </c>
       <c r="R40" t="n">
         <v>-0.0409329177050338</v>
@@ -3168,26 +3170,26 @@
         <v>1117.260009765625</v>
       </c>
       <c r="H42" t="n">
-        <v>48.49579664481703</v>
+        <v>39.59936870471272</v>
       </c>
       <c r="I42" t="n">
-        <v>23.03828552293782</v>
+        <v>28.21408639357071</v>
       </c>
       <c r="J42" t="n">
-        <v>0.131297249416838</v>
+        <v>0.2757999568288067</v>
       </c>
       <c r="K42" t="n">
-        <v>0.3166664109605854</v>
+        <v>0.3498595136264862</v>
       </c>
       <c r="L42" t="n">
-        <v>-0.2160291876285653</v>
+        <v>0.1595846747175431</v>
       </c>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="n">
-        <v>0.2608527131782945</v>
+        <v>0.2209914151204652</v>
       </c>
       <c r="R42" t="n">
         <v>-0.0553549599522092</v>
@@ -3235,34 +3237,34 @@
         <v>491.6400146484375</v>
       </c>
       <c r="H43" t="n">
-        <v>22.6466030267598</v>
+        <v>23.70498797939785</v>
       </c>
       <c r="I43" t="n">
-        <v>21.70921678926872</v>
+        <v>20.73993942016444</v>
       </c>
       <c r="J43" t="n">
-        <v>0.09388370454060641</v>
+        <v>-0.0242781548766349</v>
       </c>
       <c r="K43" t="n">
-        <v>0.06685054898198479</v>
+        <v>0.0638164727185577</v>
       </c>
       <c r="L43" t="n">
-        <v>-0.08539542145574711</v>
+        <v>-0.1457652322493625</v>
       </c>
       <c r="M43" t="n">
-        <v>2.304098534720747</v>
+        <v>2.38225930398507</v>
       </c>
       <c r="N43" t="n">
-        <v>2.375026544913994</v>
+        <v>2.455593369195301</v>
       </c>
       <c r="O43" t="n">
-        <v>0.2366644968995169</v>
+        <v>0.1939771831854465</v>
       </c>
       <c r="P43" t="n">
-        <v>0.2470407323963809</v>
+        <v>0.2024818510174158</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.624078134343233</v>
+        <v>0.6574170665553933</v>
       </c>
       <c r="R43" t="n">
         <v>-0.2895375510860729</v>
@@ -3365,30 +3367,34 @@
         <v>165.9100036621094</v>
       </c>
       <c r="H45" t="n">
-        <v>27.19903075420673</v>
+        <v>31.71756367103404</v>
       </c>
       <c r="I45" t="n">
-        <v>6.09984984984985</v>
-      </c>
-      <c r="J45" t="inlineStr"/>
+        <v>5.230855855855856</v>
+      </c>
+      <c r="J45" t="n">
+        <v>-0.0850969396137979</v>
+      </c>
       <c r="K45" t="n">
-        <v>0.1302709636042969</v>
-      </c>
-      <c r="L45" t="inlineStr"/>
+        <v>0.1113730818414322</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.1849118697548122</v>
+      </c>
       <c r="M45" t="n">
-        <v>2.122620852282298</v>
+        <v>2.057805355976486</v>
       </c>
       <c r="N45" t="n">
-        <v>2.681825837965302</v>
+        <v>2.599934683213586</v>
       </c>
       <c r="O45" t="n">
-        <v>0.087992436180271</v>
+        <v>0.129845572013867</v>
       </c>
       <c r="P45" t="n">
-        <v>0.082059722548789</v>
+        <v>0.1210909945920526</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.4806153846153846</v>
+        <v>0.566200215285253</v>
       </c>
       <c r="R45" t="n">
         <v>-0.064821598346295</v>
@@ -3436,30 +3442,30 @@
         <v>120.5999984741211</v>
       </c>
       <c r="H46" t="n">
-        <v>16.33193799868672</v>
+        <v>33.3657746198128</v>
       </c>
       <c r="I46" t="n">
-        <v>7.384304207119741</v>
+        <v>3.614482200647249</v>
       </c>
       <c r="J46" t="n">
-        <v>-0.4296676445891084</v>
+        <v>0.2123201305672148</v>
       </c>
       <c r="K46" t="n">
-        <v>0.2807832520650351</v>
+        <v>0.1358563435105218</v>
       </c>
       <c r="L46" t="n">
-        <v>-0.4950558580286084</v>
+        <v>0.16321579959342</v>
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="n">
-        <v>0.1931914095470318</v>
+        <v>0.2206227140579574</v>
       </c>
       <c r="P46" t="n">
-        <v>0.1949680574177774</v>
+        <v>0.2226516286773404</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.4479018297359483</v>
+        <v>0.9212087297146054</v>
       </c>
       <c r="R46" t="n">
         <v>-0.03627937460181</v>
@@ -3562,26 +3568,30 @@
         <v>94.04000091552734</v>
       </c>
       <c r="H48" t="n">
-        <v>14.42787311152833</v>
+        <v>12.08863304105703</v>
       </c>
       <c r="I48" t="n">
-        <v>6.517939282428703</v>
-      </c>
-      <c r="J48" t="inlineStr"/>
+        <v>7.779208831646734</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.1272980307371156</v>
+      </c>
       <c r="K48" t="n">
-        <v>0.3125413560368785</v>
-      </c>
-      <c r="L48" t="inlineStr"/>
+        <v>0.3387006328606905</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.1300487885427494</v>
+      </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="n">
-        <v>0.1824521934758155</v>
+        <v>0.2309211348581427</v>
       </c>
       <c r="P48" t="n">
-        <v>0.2337175792507204</v>
+        <v>0.2958053154018571</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.1561044460127029</v>
+        <v>0.1307947019867549</v>
       </c>
       <c r="R48" t="n">
         <v>-0.3027876815601251</v>
@@ -3661,28 +3671,16 @@
       <c r="G50" t="n">
         <v>8.609999656677246</v>
       </c>
-      <c r="H50" t="n">
-        <v>75678166.01552096</v>
-      </c>
-      <c r="I50" t="n">
-        <v>1.137712514718104e-07</v>
-      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
-      <c r="K50" t="n">
-        <v>0.0206678215160384</v>
-      </c>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
-      <c r="O50" t="n">
-        <v>-0.040197316495659</v>
-      </c>
-      <c r="P50" t="n">
-        <v>-0.0420134792902337</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>1.014450867052023</v>
-      </c>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
       <c r="R50" t="n">
         <v>-0.1012526382832746</v>
       </c>
@@ -3823,19 +3821,19 @@
         <v>5.863761153054221</v>
       </c>
       <c r="J53" t="n">
-        <v>0.0454986877670045</v>
+        <v>0.0508275046828754</v>
       </c>
       <c r="K53" t="n">
         <v>0.2536781626260077</v>
       </c>
       <c r="L53" t="n">
-        <v>0.2546043026432032</v>
+        <v>-0.2696897808526359</v>
       </c>
       <c r="M53" t="n">
         <v>0</v>
       </c>
       <c r="N53" t="n">
-        <v>0.2550214318608523</v>
+        <v>0.2407692307692307</v>
       </c>
       <c r="O53" t="n">
         <v>-0.557212759951068</v>
@@ -3892,26 +3890,26 @@
         <v>117.0299987792969</v>
       </c>
       <c r="H54" t="n">
-        <v>25.97930017518359</v>
+        <v>24.92795692899886</v>
       </c>
       <c r="I54" t="n">
-        <v>4.504740235115662</v>
+        <v>4.694728858551384</v>
       </c>
       <c r="J54" t="n">
-        <v>0.0701974289742202</v>
+        <v>0.1252455565508865</v>
       </c>
       <c r="K54" t="n">
-        <v>0.0835231747103161</v>
+        <v>0.08913015306195909</v>
       </c>
       <c r="L54" t="n">
-        <v>0.0255107677780255</v>
+        <v>0.0189765866005253</v>
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="n">
-        <v>0.9542469904874148</v>
+        <v>0.5773424878836834</v>
       </c>
       <c r="R54" t="n">
         <v>-0.1126024078988412</v>
@@ -3959,34 +3957,34 @@
         <v>142.2700042724609</v>
       </c>
       <c r="H55" t="n">
-        <v>23.67138056523592</v>
+        <v>22.33507109327196</v>
       </c>
       <c r="I55" t="n">
-        <v>6.01021152443472</v>
+        <v>6.36980306345733</v>
       </c>
       <c r="J55" t="n">
-        <v>-0.0566304268067195</v>
+        <v>0.0322294793333419</v>
       </c>
       <c r="K55" t="n">
-        <v>0.0877295714665956</v>
+        <v>0.0914938867877086</v>
       </c>
       <c r="L55" t="n">
-        <v>-0.0988613786160413</v>
+        <v>0.0057601845087889</v>
       </c>
       <c r="M55" t="n">
-        <v>3.100608736370326</v>
+        <v>2.96418750399693</v>
       </c>
       <c r="N55" t="n">
-        <v>3.886681383370125</v>
+        <v>3.715674362089915</v>
       </c>
       <c r="O55" t="n">
-        <v>0.1132666017066761</v>
+        <v>0.1305400537396285</v>
       </c>
       <c r="P55" t="n">
-        <v>0.1111722938704535</v>
+        <v>0.1281263584987683</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.9269417475728156</v>
+        <v>0.8842322226039162</v>
       </c>
       <c r="R55" t="n">
         <v>-0.1703405189109594</v>
@@ -4034,27 +4032,27 @@
         <v>24.04000091552734</v>
       </c>
       <c r="H56" t="n">
-        <v>17.72915265048092</v>
+        <v>18.39183623640197</v>
       </c>
       <c r="I56" t="n">
-        <v>1.355958820450183</v>
+        <v>1.307101727447217</v>
       </c>
       <c r="J56" t="n">
-        <v>-0.276777342467373</v>
+        <v>-0.0355710003829496</v>
       </c>
       <c r="K56" t="n">
-        <v>0.1241790376963518</v>
+        <v>0.1183131959251362</v>
       </c>
       <c r="L56" t="n">
-        <v>-0.329009730939248</v>
+        <v>-0.0577770379929784</v>
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
       <c r="O56" t="n">
-        <v>0.09643893263621001</v>
+        <v>0.1007746995249784</v>
       </c>
       <c r="P56" t="n">
-        <v>0.0906149836743252</v>
+        <v>0.0946889135188569</v>
       </c>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="n">
@@ -4109,7 +4107,7 @@
         <v>6.850111303487509</v>
       </c>
       <c r="J57" t="n">
-        <v>0.09960622425952589</v>
+        <v>0.0558928824833768</v>
       </c>
       <c r="K57" t="n">
         <v>0.191623326452714</v>
@@ -4380,12 +4378,8 @@
       <c r="G63" t="n">
         <v>0.9810000061988832</v>
       </c>
-      <c r="H63" t="n">
-        <v>1142.932398322827</v>
-      </c>
-      <c r="I63" t="n">
-        <v>0.0008583184864112</v>
-      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
@@ -4440,30 +4434,30 @@
         <v>392.1400146484375</v>
       </c>
       <c r="H64" t="n">
-        <v>20.32286661649423</v>
+        <v>20.19378841343853</v>
       </c>
       <c r="I64" t="n">
-        <v>19.29550697981617</v>
+        <v>19.41884338985531</v>
       </c>
       <c r="J64" t="n">
-        <v>0.0958634013912693</v>
+        <v>0.1089955157069719</v>
       </c>
       <c r="K64" t="n">
-        <v>0.1972227070848121</v>
+        <v>0.1960085804029725</v>
       </c>
       <c r="L64" t="n">
-        <v>-0.0123252223588954</v>
+        <v>0.046870763737008</v>
       </c>
       <c r="M64" t="n">
-        <v>0.8572141075881724</v>
+        <v>0.84038837664152</v>
       </c>
       <c r="N64" t="n">
-        <v>1.079372996081225</v>
+        <v>1.058186644314054</v>
       </c>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="n">
-        <v>0.4545186350673615</v>
+        <v>0.4658979871018174</v>
       </c>
       <c r="R64" t="n">
         <v>-0.0218020108958288</v>
@@ -4511,28 +4505,26 @@
         <v>22.3700008392334</v>
       </c>
       <c r="H65" t="n">
-        <v>7.160479018689614</v>
+        <v>7.334888521174611</v>
       </c>
       <c r="I65" t="n">
-        <v>3.12409278497225</v>
-      </c>
-      <c r="J65" t="n">
-        <v>-0.0711955804875759</v>
-      </c>
+        <v>3.049807883876476</v>
+      </c>
+      <c r="J65" t="inlineStr"/>
       <c r="K65" t="n">
-        <v>0.1747182605373742</v>
+        <v>0.1693775290844714</v>
       </c>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="n">
-        <v>2.990543420351625</v>
+        <v>2.946072428271519</v>
       </c>
       <c r="N65" t="n">
-        <v>3.218544663470076</v>
+        <v>3.170683170048985</v>
       </c>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="n">
-        <v>0.3726142212909397</v>
+        <v>0.3773039055573701</v>
       </c>
       <c r="R65" t="n">
         <v>-0.2490768663396194</v>
@@ -4586,26 +4578,28 @@
         <v>7.57130320315928</v>
       </c>
       <c r="J66" t="n">
-        <v>0.1016336266018476</v>
+        <v>-0.0120945970806393</v>
       </c>
       <c r="K66" t="n">
-        <v>0.0329356747470891</v>
-      </c>
-      <c r="L66" t="inlineStr"/>
+        <v>0.0324412231967436</v>
+      </c>
+      <c r="L66" t="n">
+        <v>-0.0566085132800734</v>
+      </c>
       <c r="M66" t="n">
-        <v>1.745000605987153</v>
+        <v>1.813350125944584</v>
       </c>
       <c r="N66" t="n">
-        <v>1.88207490001212</v>
+        <v>1.955793450881612</v>
       </c>
       <c r="O66" t="n">
-        <v>0.09206637872243691</v>
+        <v>0.0984314616958399</v>
       </c>
       <c r="P66" t="n">
-        <v>0.0969429626590069</v>
+        <v>0.1036451921761728</v>
       </c>
       <c r="Q66" t="n">
-        <v>0.594900028977108</v>
+        <v>0.5966386554621849</v>
       </c>
       <c r="R66" t="n">
         <v>0.0241532019220298</v>
@@ -4652,28 +4646,16 @@
       <c r="G67" t="n">
         <v>167.7599945068359</v>
       </c>
-      <c r="H67" t="n">
-        <v>46.67135523424792</v>
-      </c>
-      <c r="I67" t="n">
-        <v>3.594495888641604</v>
-      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
-      <c r="K67" t="n">
-        <v>0.0436059522337927</v>
-      </c>
+      <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr"/>
-      <c r="N67" t="n">
-        <v>1.68567551851134</v>
-      </c>
+      <c r="N67" t="inlineStr"/>
       <c r="O67" t="inlineStr"/>
-      <c r="P67" t="n">
-        <v>0.1099768101672518</v>
-      </c>
-      <c r="Q67" t="n">
-        <v>0.1974584555229716</v>
-      </c>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
       <c r="R67" t="n">
         <v>-0.3259943807929298</v>
       </c>
@@ -4720,30 +4702,30 @@
         <v>320.739990234375</v>
       </c>
       <c r="H68" t="n">
-        <v>11.14020576768249</v>
+        <v>9.212205926773738</v>
       </c>
       <c r="I68" t="n">
-        <v>28.79120879120879</v>
+        <v>34.81684981684982</v>
       </c>
       <c r="J68" t="n">
-        <v>0.06626342836751339</v>
+        <v>0.2112729356055094</v>
       </c>
       <c r="K68" t="n">
-        <v>0.1287785696731383</v>
+        <v>0.1553675779494095</v>
       </c>
       <c r="L68" t="n">
-        <v>0.0172110637643374</v>
+        <v>0.1956310085345325</v>
       </c>
       <c r="M68" t="n">
-        <v>1.377762106252938</v>
+        <v>1.37614463489082</v>
       </c>
       <c r="N68" t="n">
-        <v>1.589327691584391</v>
+        <v>1.587461845503639</v>
       </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr"/>
       <c r="Q68" t="n">
-        <v>0.1556933842239185</v>
+        <v>0.1283534981588637</v>
       </c>
       <c r="R68" t="n">
         <v>0.0099502607082273</v>
@@ -4901,26 +4883,26 @@
         <v>60.11000061035156</v>
       </c>
       <c r="H71" t="n">
-        <v>12.34756287306429</v>
+        <v>11.9742571033944</v>
       </c>
       <c r="I71" t="n">
-        <v>4.868167202572347</v>
+        <v>5.019935691318328</v>
       </c>
       <c r="J71" t="n">
-        <v>-0.0460854297860745</v>
+        <v>0.0858856896536126</v>
       </c>
       <c r="K71" t="n">
-        <v>0.2641680625348967</v>
+        <v>0.2693024218588284</v>
       </c>
       <c r="L71" t="n">
-        <v>-0.0749842730155616</v>
+        <v>0.07432674839397931</v>
       </c>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr"/>
       <c r="Q71" t="n">
-        <v>0.4184940554821664</v>
+        <v>0.4095567512170125</v>
       </c>
       <c r="R71" t="n">
         <v>-0.0176499107794718</v>
@@ -4967,29 +4949,15 @@
       <c r="G72" t="n">
         <v>14.84000015258789</v>
       </c>
-      <c r="H72" t="n">
-        <v>13.95162781901144</v>
-      </c>
-      <c r="I72" t="n">
-        <v>1.063675174330976</v>
-      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
-      <c r="K72" t="n">
-        <v>0.1130391975878407</v>
-      </c>
+      <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr"/>
-      <c r="M72" t="n">
-        <v>2.222409868565974</v>
-      </c>
-      <c r="N72" t="n">
-        <v>2.429693810118217</v>
-      </c>
-      <c r="O72" t="n">
-        <v>0.0834290197879588</v>
-      </c>
-      <c r="P72" t="n">
-        <v>0.0859023241608291</v>
-      </c>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
       <c r="Q72" t="inlineStr"/>
       <c r="R72" t="n">
         <v>-0.172798232396071</v>
@@ -5070,28 +5038,28 @@
         <v>45.68000030517578</v>
       </c>
       <c r="H74" t="n">
-        <v>11.19790388289216</v>
+        <v>11.09070364964187</v>
       </c>
       <c r="I74" t="n">
-        <v>4.079334916864608</v>
+        <v>4.118764845605701</v>
       </c>
       <c r="J74" t="n">
-        <v>-0.0606466905474862</v>
+        <v>-0.0114206928698575</v>
       </c>
       <c r="K74" t="n">
-        <v>0.1242772684183485</v>
+        <v>0.1246173084386184</v>
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="n">
-        <v>1.956477902873467</v>
+        <v>1.932969473094403</v>
       </c>
       <c r="N74" t="n">
-        <v>2.558687615526802</v>
+        <v>2.527943221200739</v>
       </c>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
       <c r="Q74" t="n">
-        <v>0.6685105391871433</v>
+        <v>0.6652249134948097</v>
       </c>
       <c r="R74" t="n">
         <v>-0.1160990705218532</v>
@@ -5145,13 +5113,13 @@
         <v>1.671954125707477</v>
       </c>
       <c r="J75" t="n">
-        <v>-0.1071323268515644</v>
+        <v>0.0425909888750237</v>
       </c>
       <c r="K75" t="n">
         <v>0.3904338404979244</v>
       </c>
       <c r="L75" t="n">
-        <v>-0.1704721013271365</v>
+        <v>0.056042119527252</v>
       </c>
       <c r="M75" t="n">
         <v>4.000969626636484</v>
@@ -5214,34 +5182,34 @@
         <v>119</v>
       </c>
       <c r="H76" t="n">
-        <v>43.47878317270361</v>
+        <v>41.86668719211823</v>
       </c>
       <c r="I76" t="n">
-        <v>2.736967120890111</v>
+        <v>2.842355294411802</v>
       </c>
       <c r="J76" t="n">
-        <v>-0.0330923737903134</v>
+        <v>-0.1048541398667924</v>
       </c>
       <c r="K76" t="n">
-        <v>0.030698451826581</v>
+        <v>0.031346812720166</v>
       </c>
       <c r="L76" t="n">
-        <v>0.1379159209375027</v>
+        <v>0.0819053740890953</v>
       </c>
       <c r="M76" t="n">
-        <v>0.9373940808056</v>
+        <v>0.9340446880888869</v>
       </c>
       <c r="N76" t="n">
-        <v>1.295222890826477</v>
+        <v>1.290594943833974</v>
       </c>
       <c r="O76" t="n">
-        <v>0.1126298152397053</v>
+        <v>0.09473493539427599</v>
       </c>
       <c r="P76" t="n">
-        <v>0.1094575167233892</v>
+        <v>0.09206665884285881</v>
       </c>
       <c r="Q76" t="n">
-        <v>0.3428949892659754</v>
+        <v>0.3342276565798733</v>
       </c>
       <c r="R76" t="n">
         <v>-0.119562024447027</v>
@@ -5289,30 +5257,26 @@
         <v>136.8999938964844</v>
       </c>
       <c r="H77" t="n">
-        <v>20.97354989004869</v>
+        <v>23.89828051783853</v>
       </c>
       <c r="I77" t="n">
-        <v>6.527268612808328</v>
-      </c>
-      <c r="J77" t="n">
-        <v>0.1274476553785779</v>
-      </c>
+        <v>5.728445349626613</v>
+      </c>
+      <c r="J77" t="inlineStr"/>
       <c r="K77" t="n">
-        <v>0.08681728158729581</v>
-      </c>
-      <c r="L77" t="n">
-        <v>0.0466058868699388</v>
-      </c>
+        <v>0.0757346385596237</v>
+      </c>
+      <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="n">
-        <v>0.0850941145519873</v>
+        <v>0.067723555847067</v>
       </c>
       <c r="P77" t="n">
-        <v>0.0814833475396598</v>
+        <v>0.0648498673117604</v>
       </c>
       <c r="Q77" t="n">
-        <v>0.5973859381500486</v>
+        <v>0.6806510231492455</v>
       </c>
       <c r="R77" t="n">
         <v>-0.2239669460089198</v>
@@ -5361,22 +5325,20 @@
       </c>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="n">
-        <v>-8.166472226851742</v>
+        <v>-8.285517011499726</v>
       </c>
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="n">
-        <v>-0.1465394474508687</v>
-      </c>
-      <c r="L78" t="n">
-        <v>-0.5718737669782932</v>
-      </c>
+        <v>-0.1408716772365403</v>
+      </c>
+      <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="n">
-        <v>0.0408296943231441</v>
+        <v>0.0272925764192139</v>
       </c>
       <c r="P78" t="n">
-        <v>0.0425871099977226</v>
+        <v>0.0284673195171942</v>
       </c>
       <c r="Q78" t="inlineStr"/>
       <c r="R78" t="n">
@@ -5415,7 +5377,7 @@
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
@@ -5558,7 +5520,7 @@
         <v>8508000000</v>
       </c>
       <c r="H3" t="n">
-        <v>8788000000</v>
+        <v>8743000000</v>
       </c>
       <c r="I3" t="n">
         <v>5343000000</v>
@@ -5582,7 +5544,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>DepreciationAndAmortization</t>
+          <t>DepreciationDepletionAndAmortization</t>
         </is>
       </c>
     </row>
@@ -5607,16 +5569,16 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>36751000000</v>
+        <v>37220000000</v>
       </c>
       <c r="G4" t="n">
-        <v>7711000000</v>
+        <v>7800000000</v>
       </c>
       <c r="H4" t="n">
-        <v>14247000000</v>
+        <v>15464000000</v>
       </c>
       <c r="I4" t="n">
-        <v>8100000000</v>
+        <v>8597000000</v>
       </c>
       <c r="J4" t="n">
         <v>544000000</v>
@@ -5662,14 +5624,14 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>8855500000</v>
+        <v>9005700000</v>
       </c>
       <c r="G5" t="n">
-        <v>688000000</v>
+        <v>689800000</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>712400000</v>
+        <v>872900000</v>
       </c>
       <c r="J5" t="n">
         <v>77000000</v>
@@ -5715,14 +5677,14 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>41304000000</v>
+        <v>42195000000</v>
       </c>
       <c r="G6" t="n">
-        <v>10833000000</v>
+        <v>11220000000</v>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>16003000000</v>
+        <v>14324000000</v>
       </c>
       <c r="J6" t="n">
         <v>686000000</v>
@@ -5764,10 +5726,10 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>113097000000</v>
+        <v>115122000000</v>
       </c>
       <c r="G7" t="n">
-        <v>30509000000</v>
+        <v>31733000000</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -5853,7 +5815,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>-879000000</v>
+        <v>-1161000000</v>
       </c>
       <c r="J9" t="n">
         <v>195733665</v>
@@ -5899,7 +5861,9 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>11143000000</v>
+      </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -5930,16 +5894,16 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>9890600000</v>
+        <v>9937400000</v>
       </c>
       <c r="G11" t="n">
-        <v>1292900000</v>
+        <v>1371900000</v>
       </c>
       <c r="H11" t="n">
-        <v>3620600000</v>
+        <v>3278600000</v>
       </c>
       <c r="I11" t="n">
-        <v>2050800000</v>
+        <v>2422900000</v>
       </c>
       <c r="J11" t="n">
         <v>148400000</v>
@@ -6065,16 +6029,16 @@
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
-        <v>67589000000</v>
+        <v>70755000000</v>
       </c>
       <c r="G14" t="n">
-        <v>8882000000</v>
+        <v>9427000000</v>
       </c>
       <c r="H14" t="n">
-        <v>13413000000</v>
+        <v>13974000000</v>
       </c>
       <c r="I14" t="n">
-        <v>8918000000</v>
+        <v>9481000000</v>
       </c>
       <c r="J14" t="n">
         <v>465800000</v>
@@ -6118,16 +6082,16 @@
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>20382000000</v>
+        <v>20795000000</v>
       </c>
       <c r="G15" t="n">
-        <v>2132000000</v>
+        <v>2088000000</v>
       </c>
       <c r="H15" t="n">
-        <v>3936000000</v>
+        <v>3832000000</v>
       </c>
       <c r="I15" t="n">
-        <v>3634000000</v>
+        <v>3767000000</v>
       </c>
       <c r="J15" t="n">
         <v>805100000</v>
@@ -6283,16 +6247,16 @@
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
-        <v>11100000000</v>
+        <v>11604000000</v>
       </c>
       <c r="G18" t="n">
-        <v>2031000000</v>
+        <v>2044000000</v>
       </c>
       <c r="H18" t="n">
-        <v>2684000000</v>
+        <v>2698000000</v>
       </c>
       <c r="I18" t="n">
-        <v>1434000000</v>
+        <v>1687000000</v>
       </c>
       <c r="J18" t="n">
         <v>457000000</v>
@@ -6313,7 +6277,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>DepreciationAndAmortization</t>
+          <t>DepreciationDepletionAndAmortization</t>
         </is>
       </c>
     </row>
@@ -6369,16 +6333,16 @@
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>45855000000</v>
+        <v>48312000000</v>
       </c>
       <c r="G20" t="n">
-        <v>8704000000</v>
+        <v>8630000000</v>
       </c>
       <c r="H20" t="n">
-        <v>27839000000</v>
+        <v>31426000000</v>
       </c>
       <c r="I20" t="n">
-        <v>7264000000</v>
+        <v>7455000000</v>
       </c>
       <c r="J20" t="n">
         <v>1054000000</v>
@@ -6399,7 +6363,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>DepreciationDepletionAndAmortization</t>
         </is>
       </c>
     </row>
@@ -6424,16 +6388,16 @@
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>7245519000</v>
+        <v>7463909000</v>
       </c>
       <c r="G21" t="n">
-        <v>1663887000</v>
+        <v>1736196000</v>
       </c>
       <c r="H21" t="n">
-        <v>2028687000</v>
+        <v>2162851000</v>
       </c>
       <c r="I21" t="n">
-        <v>1362913000</v>
+        <v>1451558000</v>
       </c>
       <c r="J21" t="n">
         <v>193565000</v>
@@ -6476,11 +6440,11 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
-        <v>17176000000</v>
+        <v>18068000000</v>
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
-        <v>-47218000000</v>
+        <v>-41922000000</v>
       </c>
       <c r="J22" t="n">
         <v>308000000</v>
@@ -6553,16 +6517,16 @@
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>164683000000</v>
+        <v>166592000000</v>
       </c>
       <c r="G24" t="n">
-        <v>14156000000</v>
+        <v>14012000000</v>
       </c>
       <c r="H24" t="n">
-        <v>24404000000</v>
+        <v>24307000000</v>
       </c>
       <c r="I24" t="n">
-        <v>12646000000</v>
+        <v>14315000000</v>
       </c>
       <c r="J24" t="n">
         <v>996000000</v>
@@ -6647,10 +6611,10 @@
         <v>4101000000</v>
       </c>
       <c r="H26" t="n">
-        <v>9515000000</v>
+        <v>9674000000</v>
       </c>
       <c r="I26" t="n">
-        <v>5422000000</v>
+        <v>4142000000</v>
       </c>
       <c r="J26" t="n">
         <v>638400000</v>
@@ -6751,16 +6715,16 @@
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
-        <v>8252000000</v>
+        <v>8623000000</v>
       </c>
       <c r="G28" t="n">
-        <v>1508000000</v>
+        <v>1744000000</v>
       </c>
       <c r="H28" t="n">
-        <v>2329000000</v>
+        <v>2593000000</v>
       </c>
       <c r="I28" t="n">
-        <v>1431000000</v>
+        <v>1656000000</v>
       </c>
       <c r="J28" t="n">
         <v>403000000</v>
@@ -6806,14 +6770,14 @@
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="n">
-        <v>67535000000</v>
+        <v>68911000000</v>
       </c>
       <c r="G29" t="n">
-        <v>10593000000</v>
+        <v>10754000000</v>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
-        <v>12102000000</v>
+        <v>12913000000</v>
       </c>
       <c r="J29" t="n">
         <v>952131057</v>
@@ -6890,7 +6854,9 @@
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="n">
+        <v>3162000000</v>
+      </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
@@ -6952,16 +6918,16 @@
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
-        <v>52853000000</v>
+        <v>53763000000</v>
       </c>
       <c r="G33" t="n">
-        <v>-267000000</v>
+        <v>-3174000000</v>
       </c>
       <c r="H33" t="n">
-        <v>8543000000</v>
+        <v>7119000000</v>
       </c>
       <c r="I33" t="n">
-        <v>-4949000000</v>
+        <v>-3119000000</v>
       </c>
       <c r="J33" t="n">
         <v>5083000000</v>
@@ -7040,16 +7006,16 @@
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
-        <v>94193000000</v>
+        <v>96362000000</v>
       </c>
       <c r="G35" t="n">
-        <v>26804000000</v>
+        <v>21040000000</v>
       </c>
       <c r="H35" t="n">
-        <v>29093000000</v>
+        <v>29501000000</v>
       </c>
       <c r="I35" t="n">
-        <v>19698000000</v>
+        <v>17784000000</v>
       </c>
       <c r="J35" t="n">
         <v>2445200000</v>
@@ -7098,7 +7064,7 @@
         <v>182447000000</v>
       </c>
       <c r="G36" t="n">
-        <v>57048000000</v>
+        <v>58899000000</v>
       </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
@@ -7142,19 +7108,11 @@
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="n">
-        <v>-520180000</v>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="n">
-        <v>3728859000</v>
-      </c>
-      <c r="J37" t="n">
-        <v>343029000</v>
-      </c>
-      <c r="K37" t="n">
-        <v>15033199000</v>
-      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
@@ -7185,7 +7143,9 @@
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+      <c r="G38" t="n">
+        <v>2470000000</v>
+      </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -7222,10 +7182,10 @@
         <v>2119000000</v>
       </c>
       <c r="H39" t="n">
-        <v>3156000000</v>
+        <v>3253000000</v>
       </c>
       <c r="I39" t="n">
-        <v>1639000000</v>
+        <v>1837000000</v>
       </c>
       <c r="J39" t="n">
         <v>333200000</v>
@@ -7271,16 +7231,16 @@
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
-        <v>47941000000</v>
+        <v>49284000000</v>
       </c>
       <c r="G40" t="n">
-        <v>13107000000</v>
+        <v>13701000000</v>
       </c>
       <c r="H40" t="n">
-        <v>14812000000</v>
+        <v>15509000000</v>
       </c>
       <c r="I40" t="n">
-        <v>5296000000</v>
+        <v>12562000000</v>
       </c>
       <c r="J40" t="n">
         <v>4314000000</v>
@@ -7357,10 +7317,10 @@
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="n">
-        <v>65179000000</v>
+        <v>72249000000</v>
       </c>
       <c r="G42" t="n">
-        <v>20640000000</v>
+        <v>25277000000</v>
       </c>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
@@ -7408,16 +7368,16 @@
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="n">
-        <v>75048000000</v>
+        <v>75106000000</v>
       </c>
       <c r="G43" t="n">
-        <v>5017000000</v>
+        <v>4793000000</v>
       </c>
       <c r="H43" t="n">
-        <v>9418000000</v>
+        <v>9109000000</v>
       </c>
       <c r="I43" t="n">
-        <v>6908000000</v>
+        <v>5662000000</v>
       </c>
       <c r="J43" t="n">
         <v>231100000</v>
@@ -7496,16 +7456,16 @@
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="n">
-        <v>24948000000</v>
+        <v>25024000000</v>
       </c>
       <c r="G45" t="n">
-        <v>3250000000</v>
+        <v>2787000000</v>
       </c>
       <c r="H45" t="n">
-        <v>5937000000</v>
+        <v>6124000000</v>
       </c>
       <c r="I45" t="n">
-        <v>1396000000</v>
+        <v>2060000000</v>
       </c>
       <c r="J45" t="n">
         <v>532800000</v>
@@ -7551,14 +7511,14 @@
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="n">
-        <v>65011000000</v>
+        <v>65768000000</v>
       </c>
       <c r="G46" t="n">
-        <v>18254000000</v>
+        <v>8935000000</v>
       </c>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="n">
-        <v>12360000000</v>
+        <v>14115000000</v>
       </c>
       <c r="J46" t="n">
         <v>2472000000</v>
@@ -7579,7 +7539,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>DepreciationDepletionAndAmortization</t>
         </is>
       </c>
     </row>
@@ -7637,14 +7597,14 @@
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="n">
-        <v>22669000000</v>
+        <v>24966000000</v>
       </c>
       <c r="G48" t="n">
-        <v>7085000000</v>
+        <v>8456000000</v>
       </c>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="n">
-        <v>7299000000</v>
+        <v>9238000000</v>
       </c>
       <c r="J48" t="n">
         <v>1087000000</v>
@@ -7720,22 +7680,12 @@
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
-      <c r="F50" t="n">
-        <v>16741000000</v>
-      </c>
-      <c r="G50" t="n">
-        <v>346000000</v>
-      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
-      <c r="I50" t="n">
-        <v>-5093000000</v>
-      </c>
-      <c r="J50" t="n">
-        <v>3041190068000000</v>
-      </c>
-      <c r="K50" t="n">
-        <v>25166000000</v>
-      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="n">
         <v>101534000000</v>
       </c>
@@ -7805,7 +7755,9 @@
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
+      <c r="G52" t="n">
+        <v>13967000000</v>
+      </c>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
@@ -7842,7 +7794,7 @@
         <v>17087000000</v>
       </c>
       <c r="H53" t="n">
-        <v>28229000000</v>
+        <v>29900000000</v>
       </c>
       <c r="I53" t="n">
         <v>-23686000000</v>
@@ -7891,14 +7843,14 @@
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="n">
-        <v>28444800000</v>
+        <v>27779600000</v>
       </c>
       <c r="G54" t="n">
-        <v>2375800000</v>
+        <v>2476000000</v>
       </c>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="n">
-        <v>3672800000</v>
+        <v>3752200000</v>
       </c>
       <c r="J54" t="n">
         <v>527400000</v>
@@ -7940,16 +7892,16 @@
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="n">
-        <v>93925000000</v>
+        <v>95449000000</v>
       </c>
       <c r="G55" t="n">
-        <v>8240000000</v>
+        <v>8733000000</v>
       </c>
       <c r="H55" t="n">
-        <v>14949000000</v>
+        <v>15637000000</v>
       </c>
       <c r="I55" t="n">
-        <v>7672000000</v>
+        <v>8842000000</v>
       </c>
       <c r="J55" t="n">
         <v>1371000000</v>
@@ -7995,14 +7947,14 @@
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="n">
-        <v>62579000000</v>
+        <v>63315000000</v>
       </c>
       <c r="G56" t="n">
-        <v>7771000000</v>
+        <v>7491000000</v>
       </c>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="n">
-        <v>9075000000</v>
+        <v>9483000000</v>
       </c>
       <c r="J56" t="n">
         <v>5731000000</v>
@@ -8163,7 +8115,9 @@
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
+      <c r="G60" t="n">
+        <v>10249000000</v>
+      </c>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
@@ -8256,21 +8210,11 @@
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="n">
-        <v>1281000000</v>
-      </c>
-      <c r="H63" t="n">
-        <v>821000000</v>
-      </c>
-      <c r="I63" t="n">
-        <v>-890000000</v>
-      </c>
-      <c r="J63" t="n">
-        <v>1492453000000</v>
-      </c>
-      <c r="K63" t="n">
-        <v>4264000000</v>
-      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
@@ -8301,13 +8245,13 @@
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="n">
-        <v>5156100000</v>
+        <v>5221200000</v>
       </c>
       <c r="G64" t="n">
-        <v>1016900000</v>
+        <v>1023400000</v>
       </c>
       <c r="H64" t="n">
-        <v>1403500000</v>
+        <v>1431600000</v>
       </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="n">
@@ -8329,7 +8273,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>DepreciationDepletionAndAmortization</t>
         </is>
       </c>
     </row>
@@ -8354,16 +8298,16 @@
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="n">
-        <v>125648000000</v>
+        <v>126528000000</v>
       </c>
       <c r="G65" t="n">
-        <v>21953000000</v>
+        <v>21431000000</v>
       </c>
       <c r="H65" t="n">
-        <v>45048000000</v>
+        <v>45728000000</v>
       </c>
       <c r="I65" t="n">
-        <v>19442000000</v>
+        <v>18842000000</v>
       </c>
       <c r="J65" t="n">
         <v>7027000000</v>
@@ -8407,16 +8351,16 @@
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="n">
-        <v>104780000000</v>
+        <v>106377000000</v>
       </c>
       <c r="G66" t="n">
         <v>3451000000</v>
       </c>
       <c r="H66" t="n">
-        <v>8251000000</v>
+        <v>7940000000</v>
       </c>
       <c r="I66" t="n">
-        <v>2835000000</v>
+        <v>3031000000</v>
       </c>
       <c r="J66" t="n">
         <v>455800000</v>
@@ -8461,24 +8405,12 @@
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
-      <c r="F67" t="n">
-        <v>234601000000</v>
-      </c>
-      <c r="G67" t="n">
-        <v>10230000000</v>
-      </c>
-      <c r="H67" t="n">
-        <v>25795000000</v>
-      </c>
-      <c r="I67" t="n">
-        <v>16978000000</v>
-      </c>
-      <c r="J67" t="n">
-        <v>2846018000</v>
-      </c>
-      <c r="K67" t="n">
-        <v>129166000000</v>
-      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="n">
         <v>43482000000</v>
@@ -8515,13 +8447,13 @@
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="n">
-        <v>48828000000</v>
+        <v>48942000000</v>
       </c>
       <c r="G68" t="n">
-        <v>6288000000</v>
+        <v>7604000000</v>
       </c>
       <c r="H68" t="n">
-        <v>4254000000</v>
+        <v>4259000000</v>
       </c>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="n">
@@ -8568,7 +8500,9 @@
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
+      <c r="G69" t="n">
+        <v>35301100000</v>
+      </c>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr"/>
@@ -8599,7 +8533,9 @@
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
+      <c r="G70" t="n">
+        <v>303095000</v>
+      </c>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr"/>
@@ -8630,10 +8566,10 @@
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="n">
-        <v>28656000000</v>
+        <v>28986000000</v>
       </c>
       <c r="G71" t="n">
-        <v>7570000000</v>
+        <v>7806000000</v>
       </c>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr"/>
@@ -8654,11 +8590,7 @@
           <t>Revenues</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t>Depreciation</t>
-        </is>
-      </c>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8680,24 +8612,12 @@
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
-      <c r="F72" t="n">
-        <v>48753000000</v>
-      </c>
-      <c r="G72" t="n">
-        <v>5511000000</v>
-      </c>
-      <c r="H72" t="n">
-        <v>13619000000</v>
-      </c>
-      <c r="I72" t="n">
-        <v>8719000000</v>
-      </c>
-      <c r="J72" t="n">
-        <v>5181093000</v>
-      </c>
-      <c r="K72" t="n">
-        <v>74241000000</v>
-      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
       <c r="L72" t="n">
         <v>30267000000</v>
       </c>
@@ -8767,16 +8687,16 @@
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="n">
-        <v>138191000000</v>
+        <v>139146000000</v>
       </c>
       <c r="G74" t="n">
-        <v>17174000000</v>
+        <v>17340000000</v>
       </c>
       <c r="H74" t="n">
-        <v>47608000000</v>
+        <v>48187000000</v>
       </c>
       <c r="I74" t="n">
-        <v>20173000000</v>
+        <v>20375000000</v>
       </c>
       <c r="J74" t="n">
         <v>4210000000</v>
@@ -8875,16 +8795,16 @@
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="n">
-        <v>713163000000</v>
+        <v>725305000000</v>
       </c>
       <c r="G76" t="n">
-        <v>21893000000</v>
+        <v>22736000000</v>
       </c>
       <c r="H76" t="n">
-        <v>40715000000</v>
+        <v>40861000000</v>
       </c>
       <c r="I76" t="n">
-        <v>14923000000</v>
+        <v>12552000000</v>
       </c>
       <c r="J76" t="n">
         <v>7999000000</v>
@@ -8905,7 +8825,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>DepreciationAndAmortization</t>
+          <t>DepreciationDepletionAndAmortization</t>
         </is>
       </c>
     </row>
@@ -8930,14 +8850,14 @@
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="n">
-        <v>332238000000</v>
+        <v>334246000000</v>
       </c>
       <c r="G77" t="n">
-        <v>28844000000</v>
+        <v>25314000000</v>
       </c>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="n">
-        <v>23612000000</v>
+        <v>18792000000</v>
       </c>
       <c r="J77" t="n">
         <v>4419000000</v>
@@ -8983,14 +8903,14 @@
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="n">
-        <v>7022000000</v>
+        <v>7411000000</v>
       </c>
       <c r="G78" t="n">
-        <v>-1029000000</v>
+        <v>-1044000000</v>
       </c>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="n">
-        <v>187000000</v>
+        <v>125000000</v>
       </c>
       <c r="J78" t="n">
         <v>126003000</v>

</xml_diff>